<commit_message>
fix: correct two false positive basket assignments
DRK1 (Spring Water) and FRZ18 (Chocolate cake) had Y marks from the initial
--populate-baskets run where "tuna in spring water" matched DRK1 and
"Chocolate cereal" matched FRZ18 instead of their correct Pantry targets.

Corrections applied directly to baskets tab:
  DRK1: cleared healthy and neutral Y marks
  FRZ18: cleared all three Y marks
  PAN21 Springwater tuna: set healthy=Y neutral=Y
  PAN38 Chocolate flavoured cereal: set healthy=Y neutral=Y unhealthy=Y

Rebuilt ITEM_REGISTRY from corrected baskets tab.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Combined Justification 8.05.2026.xlsx
+++ b/Combined Justification 8.05.2026.xlsx
@@ -8760,13 +8760,11 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8789,9 +8787,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -8814,9 +8809,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8839,8 +8831,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>Y</t>
@@ -8868,9 +8858,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -8893,9 +8880,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -8955,7 +8939,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>Y</t>
@@ -8988,9 +8971,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -9013,9 +8993,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -9038,9 +9015,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -9063,9 +9037,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -9088,9 +9059,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -9113,9 +9081,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -9148,7 +9113,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -9171,9 +9135,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -9196,9 +9157,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -9221,9 +9179,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -9246,9 +9201,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -9271,9 +9223,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -9296,9 +9245,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -9321,9 +9267,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -9346,9 +9289,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -9413,7 +9353,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>Y</t>
@@ -9441,9 +9380,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -9466,9 +9402,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -9491,9 +9424,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -9516,9 +9446,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr"/>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -9541,7 +9468,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>Y</t>
@@ -9574,9 +9500,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -9599,9 +9522,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
-      <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -9624,9 +9544,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
-      <c r="F34" t="inlineStr"/>
-      <c r="G34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -9649,9 +9566,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr"/>
-      <c r="G35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -9674,9 +9588,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
-      <c r="F36" t="inlineStr"/>
-      <c r="G36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -9699,9 +9610,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -9724,9 +9632,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -9749,8 +9654,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
           <t>Y</t>
@@ -9778,9 +9681,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
-      <c r="F40" t="inlineStr"/>
-      <c r="G40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -9803,9 +9703,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -9828,9 +9725,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
-      <c r="F42" t="inlineStr"/>
-      <c r="G42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -9853,9 +9747,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -9878,9 +9769,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="inlineStr"/>
-      <c r="G44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -9903,9 +9791,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -9928,9 +9813,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -9953,9 +9835,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -10015,17 +9894,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -10048,9 +9916,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
-      <c r="F50" t="inlineStr"/>
-      <c r="G50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -10073,9 +9938,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
-      <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -10098,9 +9960,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
-      <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -10123,9 +9982,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr"/>
-      <c r="G53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -10148,9 +10004,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
-      <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -10173,9 +10026,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -10198,9 +10048,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -10223,9 +10070,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
-      <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -10248,9 +10092,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
-      <c r="F58" t="inlineStr"/>
-      <c r="G58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -10273,9 +10114,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr"/>
-      <c r="G59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -10298,8 +10136,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
-      <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
           <t>Y</t>
@@ -10322,10 +10158,6 @@
           <t>Protein water citrus</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr"/>
-      <c r="E61" t="inlineStr"/>
-      <c r="F61" t="inlineStr"/>
-      <c r="G61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -10348,9 +10180,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -10373,9 +10202,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr"/>
-      <c r="G63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -10398,9 +10224,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
-      <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -10423,9 +10246,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
-      <c r="F65" t="inlineStr"/>
-      <c r="G65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -10448,8 +10268,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
           <t>Y</t>
@@ -10477,9 +10295,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
-      <c r="F67" t="inlineStr"/>
-      <c r="G67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -10502,9 +10317,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
-      <c r="F68" t="inlineStr"/>
-      <c r="G68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -10527,9 +10339,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
-      <c r="F69" t="inlineStr"/>
-      <c r="G69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -10552,9 +10361,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
-      <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -10577,13 +10383,11 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -10606,9 +10410,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
-      <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -10631,9 +10432,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
-      <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -10656,9 +10454,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
-      <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -10681,9 +10476,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr"/>
-      <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -10706,9 +10498,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
-      <c r="F76" t="inlineStr"/>
-      <c r="G76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -10731,7 +10520,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
           <t>Y</t>
@@ -10764,9 +10552,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E78" t="inlineStr"/>
-      <c r="F78" t="inlineStr"/>
-      <c r="G78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -10789,9 +10574,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
-      <c r="F79" t="inlineStr"/>
-      <c r="G79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -10814,9 +10596,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
-      <c r="F80" t="inlineStr"/>
-      <c r="G80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -10839,9 +10618,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr"/>
-      <c r="F81" t="inlineStr"/>
-      <c r="G81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -10864,9 +10640,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
-      <c r="F82" t="inlineStr"/>
-      <c r="G82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -10889,7 +10662,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
         <is>
           <t>Y</t>
@@ -10922,8 +10694,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr"/>
-      <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
         <is>
           <t>Y</t>
@@ -10951,13 +10721,11 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -10980,9 +10748,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr"/>
-      <c r="F86" t="inlineStr"/>
-      <c r="G86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -11005,9 +10770,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr"/>
-      <c r="F87" t="inlineStr"/>
-      <c r="G87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -11030,9 +10792,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
-      <c r="F88" t="inlineStr"/>
-      <c r="G88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -11060,7 +10819,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
           <t>Y</t>
@@ -11088,9 +10846,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
-      <c r="F90" t="inlineStr"/>
-      <c r="G90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -11113,9 +10868,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
-      <c r="F91" t="inlineStr"/>
-      <c r="G91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -11138,9 +10890,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr"/>
-      <c r="F92" t="inlineStr"/>
-      <c r="G92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -11163,9 +10912,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
-      <c r="F93" t="inlineStr"/>
-      <c r="G93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -11188,9 +10934,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
-      <c r="F94" t="inlineStr"/>
-      <c r="G94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -11213,9 +10956,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
-      <c r="F95" t="inlineStr"/>
-      <c r="G95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -11238,9 +10978,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E96" t="inlineStr"/>
-      <c r="F96" t="inlineStr"/>
-      <c r="G96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -11268,8 +11005,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F97" t="inlineStr"/>
-      <c r="G97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -11329,9 +11064,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr"/>
-      <c r="F99" t="inlineStr"/>
-      <c r="G99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -11354,9 +11086,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E100" t="inlineStr"/>
-      <c r="F100" t="inlineStr"/>
-      <c r="G100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -11379,9 +11108,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E101" t="inlineStr"/>
-      <c r="F101" t="inlineStr"/>
-      <c r="G101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -11404,9 +11130,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E102" t="inlineStr"/>
-      <c r="F102" t="inlineStr"/>
-      <c r="G102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -11429,9 +11152,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
-      <c r="F103" t="inlineStr"/>
-      <c r="G103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -11454,9 +11174,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr"/>
-      <c r="F104" t="inlineStr"/>
-      <c r="G104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -11479,9 +11196,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E105" t="inlineStr"/>
-      <c r="F105" t="inlineStr"/>
-      <c r="G105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -11504,9 +11218,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
-      <c r="F106" t="inlineStr"/>
-      <c r="G106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -11529,9 +11240,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
-      <c r="F107" t="inlineStr"/>
-      <c r="G107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -11554,9 +11262,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
-      <c r="F108" t="inlineStr"/>
-      <c r="G108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -11579,9 +11284,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr"/>
-      <c r="F109" t="inlineStr"/>
-      <c r="G109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -11604,9 +11306,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
-      <c r="F110" t="inlineStr"/>
-      <c r="G110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -11629,9 +11328,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
-      <c r="F111" t="inlineStr"/>
-      <c r="G111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -11654,9 +11350,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
-      <c r="F112" t="inlineStr"/>
-      <c r="G112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -11679,9 +11372,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
-      <c r="F113" t="inlineStr"/>
-      <c r="G113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -11704,9 +11394,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr"/>
-      <c r="F114" t="inlineStr"/>
-      <c r="G114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -11729,9 +11416,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
-      <c r="F115" t="inlineStr"/>
-      <c r="G115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -11791,9 +11475,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E117" t="inlineStr"/>
-      <c r="F117" t="inlineStr"/>
-      <c r="G117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -11816,9 +11497,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr"/>
-      <c r="F118" t="inlineStr"/>
-      <c r="G118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -11841,9 +11519,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E119" t="inlineStr"/>
-      <c r="F119" t="inlineStr"/>
-      <c r="G119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -11866,9 +11541,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr"/>
-      <c r="F120" t="inlineStr"/>
-      <c r="G120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -11891,9 +11563,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr"/>
-      <c r="F121" t="inlineStr"/>
-      <c r="G121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -11916,8 +11585,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E122" t="inlineStr"/>
-      <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
           <t>Y</t>
@@ -11945,9 +11612,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E123" t="inlineStr"/>
-      <c r="F123" t="inlineStr"/>
-      <c r="G123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -11970,8 +11634,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E124" t="inlineStr"/>
-      <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
           <t>Y</t>
@@ -11999,9 +11661,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E125" t="inlineStr"/>
-      <c r="F125" t="inlineStr"/>
-      <c r="G125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -12024,9 +11683,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E126" t="inlineStr"/>
-      <c r="F126" t="inlineStr"/>
-      <c r="G126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -12049,9 +11705,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E127" t="inlineStr"/>
-      <c r="F127" t="inlineStr"/>
-      <c r="G127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -12074,9 +11727,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E128" t="inlineStr"/>
-      <c r="F128" t="inlineStr"/>
-      <c r="G128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -12099,9 +11749,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E129" t="inlineStr"/>
-      <c r="F129" t="inlineStr"/>
-      <c r="G129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -12124,8 +11771,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E130" t="inlineStr"/>
-      <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
           <t>Y</t>
@@ -12153,9 +11798,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E131" t="inlineStr"/>
-      <c r="F131" t="inlineStr"/>
-      <c r="G131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -12215,9 +11857,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E133" t="inlineStr"/>
-      <c r="F133" t="inlineStr"/>
-      <c r="G133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -12240,9 +11879,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E134" t="inlineStr"/>
-      <c r="F134" t="inlineStr"/>
-      <c r="G134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -12270,8 +11906,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F135" t="inlineStr"/>
-      <c r="G135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -12294,9 +11928,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E136" t="inlineStr"/>
-      <c r="F136" t="inlineStr"/>
-      <c r="G136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -12319,9 +11950,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E137" t="inlineStr"/>
-      <c r="F137" t="inlineStr"/>
-      <c r="G137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -12344,9 +11972,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E138" t="inlineStr"/>
-      <c r="F138" t="inlineStr"/>
-      <c r="G138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -12369,9 +11994,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E139" t="inlineStr"/>
-      <c r="F139" t="inlineStr"/>
-      <c r="G139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -12394,9 +12016,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E140" t="inlineStr"/>
-      <c r="F140" t="inlineStr"/>
-      <c r="G140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -12419,9 +12038,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E141" t="inlineStr"/>
-      <c r="F141" t="inlineStr"/>
-      <c r="G141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -12444,13 +12060,11 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E142" t="inlineStr"/>
       <c r="F142" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -12473,9 +12087,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E143" t="inlineStr"/>
-      <c r="F143" t="inlineStr"/>
-      <c r="G143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -12498,13 +12109,11 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E144" t="inlineStr"/>
       <c r="F144" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="G144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -12527,9 +12136,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E145" t="inlineStr"/>
-      <c r="F145" t="inlineStr"/>
-      <c r="G145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -12552,9 +12158,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E146" t="inlineStr"/>
-      <c r="F146" t="inlineStr"/>
-      <c r="G146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -12577,9 +12180,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E147" t="inlineStr"/>
-      <c r="F147" t="inlineStr"/>
-      <c r="G147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -12602,9 +12202,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E148" t="inlineStr"/>
-      <c r="F148" t="inlineStr"/>
-      <c r="G148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -12627,21 +12224,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E149" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F149" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G149" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -12664,9 +12246,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E150" t="inlineStr"/>
-      <c r="F150" t="inlineStr"/>
-      <c r="G150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -12689,9 +12268,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E151" t="inlineStr"/>
-      <c r="F151" t="inlineStr"/>
-      <c r="G151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -12714,9 +12290,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E152" t="inlineStr"/>
-      <c r="F152" t="inlineStr"/>
-      <c r="G152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -12739,9 +12312,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E153" t="inlineStr"/>
-      <c r="F153" t="inlineStr"/>
-      <c r="G153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -12764,9 +12334,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E154" t="inlineStr"/>
-      <c r="F154" t="inlineStr"/>
-      <c r="G154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -12826,9 +12393,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E156" t="inlineStr"/>
-      <c r="F156" t="inlineStr"/>
-      <c r="G156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -12851,9 +12415,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E157" t="inlineStr"/>
-      <c r="F157" t="inlineStr"/>
-      <c r="G157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -12876,9 +12437,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E158" t="inlineStr"/>
-      <c r="F158" t="inlineStr"/>
-      <c r="G158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -12901,9 +12459,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E159" t="inlineStr"/>
-      <c r="F159" t="inlineStr"/>
-      <c r="G159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -12926,9 +12481,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E160" t="inlineStr"/>
-      <c r="F160" t="inlineStr"/>
-      <c r="G160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -12956,8 +12508,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F161" t="inlineStr"/>
-      <c r="G161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -12980,9 +12530,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E162" t="inlineStr"/>
-      <c r="F162" t="inlineStr"/>
-      <c r="G162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -13005,9 +12552,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E163" t="inlineStr"/>
-      <c r="F163" t="inlineStr"/>
-      <c r="G163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -13030,9 +12574,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E164" t="inlineStr"/>
-      <c r="F164" t="inlineStr"/>
-      <c r="G164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -13055,9 +12596,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E165" t="inlineStr"/>
-      <c r="F165" t="inlineStr"/>
-      <c r="G165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -13080,9 +12618,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E166" t="inlineStr"/>
-      <c r="F166" t="inlineStr"/>
-      <c r="G166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -13105,9 +12640,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E167" t="inlineStr"/>
-      <c r="F167" t="inlineStr"/>
-      <c r="G167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -13130,9 +12662,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E168" t="inlineStr"/>
-      <c r="F168" t="inlineStr"/>
-      <c r="G168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -13160,8 +12689,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F169" t="inlineStr"/>
-      <c r="G169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -13184,9 +12711,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E170" t="inlineStr"/>
-      <c r="F170" t="inlineStr"/>
-      <c r="G170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -13209,9 +12733,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E171" t="inlineStr"/>
-      <c r="F171" t="inlineStr"/>
-      <c r="G171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -13234,9 +12755,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E172" t="inlineStr"/>
-      <c r="F172" t="inlineStr"/>
-      <c r="G172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -13259,9 +12777,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E173" t="inlineStr"/>
-      <c r="F173" t="inlineStr"/>
-      <c r="G173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -13284,9 +12799,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E174" t="inlineStr"/>
-      <c r="F174" t="inlineStr"/>
-      <c r="G174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -13309,9 +12821,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E175" t="inlineStr"/>
-      <c r="F175" t="inlineStr"/>
-      <c r="G175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -13334,9 +12843,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E176" t="inlineStr"/>
-      <c r="F176" t="inlineStr"/>
-      <c r="G176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -13359,9 +12865,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E177" t="inlineStr"/>
-      <c r="F177" t="inlineStr"/>
-      <c r="G177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -13384,9 +12887,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E178" t="inlineStr"/>
-      <c r="F178" t="inlineStr"/>
-      <c r="G178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -13409,9 +12909,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E179" t="inlineStr"/>
-      <c r="F179" t="inlineStr"/>
-      <c r="G179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -13434,9 +12931,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E180" t="inlineStr"/>
-      <c r="F180" t="inlineStr"/>
-      <c r="G180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -13459,9 +12953,16 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E181" t="inlineStr"/>
-      <c r="F181" t="inlineStr"/>
-      <c r="G181" t="inlineStr"/>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -13484,9 +12985,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E182" t="inlineStr"/>
-      <c r="F182" t="inlineStr"/>
-      <c r="G182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -13509,9 +13007,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E183" t="inlineStr"/>
-      <c r="F183" t="inlineStr"/>
-      <c r="G183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -13534,9 +13029,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E184" t="inlineStr"/>
-      <c r="F184" t="inlineStr"/>
-      <c r="G184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -13564,8 +13056,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F185" t="inlineStr"/>
-      <c r="G185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -13588,9 +13078,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E186" t="inlineStr"/>
-      <c r="F186" t="inlineStr"/>
-      <c r="G186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -13613,9 +13100,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E187" t="inlineStr"/>
-      <c r="F187" t="inlineStr"/>
-      <c r="G187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -13638,9 +13122,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E188" t="inlineStr"/>
-      <c r="F188" t="inlineStr"/>
-      <c r="G188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -13663,9 +13144,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E189" t="inlineStr"/>
-      <c r="F189" t="inlineStr"/>
-      <c r="G189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -13688,9 +13166,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E190" t="inlineStr"/>
-      <c r="F190" t="inlineStr"/>
-      <c r="G190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -13713,9 +13188,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E191" t="inlineStr"/>
-      <c r="F191" t="inlineStr"/>
-      <c r="G191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -13738,9 +13210,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E192" t="inlineStr"/>
-      <c r="F192" t="inlineStr"/>
-      <c r="G192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -13763,9 +13232,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E193" t="inlineStr"/>
-      <c r="F193" t="inlineStr"/>
-      <c r="G193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -13788,9 +13254,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E194" t="inlineStr"/>
-      <c r="F194" t="inlineStr"/>
-      <c r="G194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -13813,9 +13276,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E195" t="inlineStr"/>
-      <c r="F195" t="inlineStr"/>
-      <c r="G195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -13838,9 +13298,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E196" t="inlineStr"/>
-      <c r="F196" t="inlineStr"/>
-      <c r="G196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -13863,9 +13320,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E197" t="inlineStr"/>
-      <c r="F197" t="inlineStr"/>
-      <c r="G197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -13888,9 +13342,21 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E198" t="inlineStr"/>
-      <c r="F198" t="inlineStr"/>
-      <c r="G198" t="inlineStr"/>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F198" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -13913,9 +13379,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E199" t="inlineStr"/>
-      <c r="F199" t="inlineStr"/>
-      <c r="G199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -13938,9 +13401,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E200" t="inlineStr"/>
-      <c r="F200" t="inlineStr"/>
-      <c r="G200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -13963,9 +13423,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E201" t="inlineStr"/>
-      <c r="F201" t="inlineStr"/>
-      <c r="G201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -13988,9 +13445,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E202" t="inlineStr"/>
-      <c r="F202" t="inlineStr"/>
-      <c r="G202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -14013,8 +13467,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E203" t="inlineStr"/>
-      <c r="F203" t="inlineStr"/>
       <c r="G203" t="inlineStr">
         <is>
           <t>Y</t>
@@ -14042,8 +13494,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E204" t="inlineStr"/>
-      <c r="F204" t="inlineStr"/>
       <c r="G204" t="inlineStr">
         <is>
           <t>Y</t>
@@ -14071,9 +13521,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E205" t="inlineStr"/>
-      <c r="F205" t="inlineStr"/>
-      <c r="G205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -14096,9 +13543,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E206" t="inlineStr"/>
-      <c r="F206" t="inlineStr"/>
-      <c r="G206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -14121,9 +13565,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E207" t="inlineStr"/>
-      <c r="F207" t="inlineStr"/>
-      <c r="G207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -14146,9 +13587,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E208" t="inlineStr"/>
-      <c r="F208" t="inlineStr"/>
-      <c r="G208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -14171,9 +13609,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E209" t="inlineStr"/>
-      <c r="F209" t="inlineStr"/>
-      <c r="G209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -14196,9 +13631,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E210" t="inlineStr"/>
-      <c r="F210" t="inlineStr"/>
-      <c r="G210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -14221,9 +13653,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E211" t="inlineStr"/>
-      <c r="F211" t="inlineStr"/>
-      <c r="G211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -14246,9 +13675,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E212" t="inlineStr"/>
-      <c r="F212" t="inlineStr"/>
-      <c r="G212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -14271,9 +13697,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E213" t="inlineStr"/>
-      <c r="F213" t="inlineStr"/>
-      <c r="G213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -14306,7 +13729,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -14329,9 +13751,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E215" t="inlineStr"/>
-      <c r="F215" t="inlineStr"/>
-      <c r="G215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -14354,7 +13773,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E216" t="inlineStr"/>
       <c r="F216" t="inlineStr">
         <is>
           <t>Y</t>
@@ -14387,8 +13805,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E217" t="inlineStr"/>
-      <c r="F217" t="inlineStr"/>
       <c r="G217" t="inlineStr">
         <is>
           <t>Y</t>
@@ -14416,9 +13832,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E218" t="inlineStr"/>
-      <c r="F218" t="inlineStr"/>
-      <c r="G218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -14441,9 +13854,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E219" t="inlineStr"/>
-      <c r="F219" t="inlineStr"/>
-      <c r="G219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -14466,8 +13876,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E220" t="inlineStr"/>
-      <c r="F220" t="inlineStr"/>
       <c r="G220" t="inlineStr">
         <is>
           <t>Y</t>
@@ -14495,9 +13903,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E221" t="inlineStr"/>
-      <c r="F221" t="inlineStr"/>
-      <c r="G221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -14520,9 +13925,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E222" t="inlineStr"/>
-      <c r="F222" t="inlineStr"/>
-      <c r="G222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -14545,9 +13947,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E223" t="inlineStr"/>
-      <c r="F223" t="inlineStr"/>
-      <c r="G223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -14570,9 +13969,6 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="E224" t="inlineStr"/>
-      <c r="F224" t="inlineStr"/>
-      <c r="G224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -14595,9 +13991,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E225" t="inlineStr"/>
-      <c r="F225" t="inlineStr"/>
-      <c r="G225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -14630,7 +14023,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -14653,9 +14045,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E227" t="inlineStr"/>
-      <c r="F227" t="inlineStr"/>
-      <c r="G227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -14688,7 +14077,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -14711,9 +14099,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E229" t="inlineStr"/>
-      <c r="F229" t="inlineStr"/>
-      <c r="G229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -14746,7 +14131,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -14779,7 +14163,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -14802,9 +14185,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E232" t="inlineStr"/>
-      <c r="F232" t="inlineStr"/>
-      <c r="G232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -14827,9 +14207,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E233" t="inlineStr"/>
-      <c r="F233" t="inlineStr"/>
-      <c r="G233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -14857,8 +14234,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F234" t="inlineStr"/>
-      <c r="G234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -14881,9 +14256,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E235" t="inlineStr"/>
-      <c r="F235" t="inlineStr"/>
-      <c r="G235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -14906,9 +14278,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E236" t="inlineStr"/>
-      <c r="F236" t="inlineStr"/>
-      <c r="G236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -14931,9 +14300,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E237" t="inlineStr"/>
-      <c r="F237" t="inlineStr"/>
-      <c r="G237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -14961,8 +14327,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F238" t="inlineStr"/>
-      <c r="G238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -14985,9 +14349,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E239" t="inlineStr"/>
-      <c r="F239" t="inlineStr"/>
-      <c r="G239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -15010,9 +14371,6 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E240" t="inlineStr"/>
-      <c r="F240" t="inlineStr"/>
-      <c r="G240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -15045,7 +14403,6 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="G241" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
checkpoint: commit updated Excel files
Combined Justification and bakery_dairy_overrides updated by build pipeline
runs this session.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Combined Justification 8.05.2026.xlsx
+++ b/Combined Justification 8.05.2026.xlsx
@@ -8710,11 +8710,13 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8737,6 +8739,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -8759,6 +8764,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8781,6 +8789,8 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>Y</t>
@@ -8808,6 +8818,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -8830,6 +8843,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -8889,6 +8905,7 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>Y</t>
@@ -8921,6 +8938,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -8943,6 +8963,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -8965,6 +8988,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -8987,6 +9013,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -9009,6 +9038,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -9031,6 +9063,13 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -9053,16 +9092,13 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -9085,6 +9121,13 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -9107,6 +9150,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -9129,6 +9175,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -9151,6 +9200,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -9173,6 +9225,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -9195,6 +9250,13 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -9217,6 +9279,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -9239,6 +9304,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -9303,6 +9371,7 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" t="inlineStr">
         <is>
           <t>Y</t>
@@ -9330,6 +9399,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E27" t="inlineStr"/>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -9352,6 +9424,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E28" t="inlineStr"/>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -9374,6 +9449,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -9396,6 +9474,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -9418,6 +9499,7 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>Y</t>
@@ -9450,6 +9532,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
+      <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -9472,6 +9557,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -9494,6 +9582,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -9516,6 +9607,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -9538,6 +9632,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr"/>
+      <c r="G36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -9560,6 +9657,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -9582,6 +9682,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -9604,6 +9707,8 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
       <c r="G39" t="inlineStr">
         <is>
           <t>Y</t>
@@ -9631,6 +9736,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -9653,6 +9761,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -9675,6 +9786,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -9697,6 +9811,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E43" t="inlineStr"/>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -9719,6 +9836,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -9741,6 +9861,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E45" t="inlineStr"/>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -9763,6 +9886,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -9785,6 +9911,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E47" t="inlineStr"/>
+      <c r="F47" t="inlineStr"/>
+      <c r="G47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -9844,6 +9973,17 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -9866,6 +10006,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E50" t="inlineStr"/>
+      <c r="F50" t="inlineStr"/>
+      <c r="G50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -9888,6 +10031,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E51" t="inlineStr"/>
+      <c r="F51" t="inlineStr"/>
+      <c r="G51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -9910,6 +10056,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E52" t="inlineStr"/>
+      <c r="F52" t="inlineStr"/>
+      <c r="G52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -9932,6 +10081,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -9954,6 +10106,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E54" t="inlineStr"/>
+      <c r="F54" t="inlineStr"/>
+      <c r="G54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -9976,6 +10131,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -9998,6 +10156,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -10012,7 +10173,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Energy Drink</t>
+          <t>Energy drink</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -10020,6 +10181,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E57" t="inlineStr"/>
+      <c r="F57" t="inlineStr"/>
+      <c r="G57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -10042,6 +10206,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E58" t="inlineStr"/>
+      <c r="F58" t="inlineStr"/>
+      <c r="G58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -10064,6 +10231,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E59" t="inlineStr"/>
+      <c r="F59" t="inlineStr"/>
+      <c r="G59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -10086,6 +10256,8 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E60" t="inlineStr"/>
+      <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
           <t>Y</t>
@@ -10108,6 +10280,10 @@
           <t>Protein water citrus</t>
         </is>
       </c>
+      <c r="D61" t="inlineStr"/>
+      <c r="E61" t="inlineStr"/>
+      <c r="F61" t="inlineStr"/>
+      <c r="G61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -10130,6 +10306,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E62" t="inlineStr"/>
+      <c r="F62" t="inlineStr"/>
+      <c r="G62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -10144,7 +10323,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Wholegrain rice crackers</t>
+          <t>Wholegrain rice cracker</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -10152,6 +10331,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -10166,7 +10348,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Multigrain crispbread crackers</t>
+          <t>Multigrain crispbread cracker</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -10174,6 +10356,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -10188,7 +10373,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Mini rice crisps milk chocolate</t>
+          <t>Rice crisps milk chocolate</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -10196,6 +10381,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E65" t="inlineStr"/>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -10218,6 +10406,8 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E66" t="inlineStr"/>
+      <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr">
         <is>
           <t>Y</t>
@@ -10245,6 +10435,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E67" t="inlineStr"/>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -10259,7 +10452,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Jelly beans</t>
+          <t>Jelly bean</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -10267,6 +10460,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E68" t="inlineStr"/>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -10289,6 +10485,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E69" t="inlineStr"/>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -10303,7 +10502,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Marshmallows</t>
+          <t>Marshmallow</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -10311,6 +10510,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E70" t="inlineStr"/>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -10333,11 +10535,13 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
+      <c r="G71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -10360,6 +10564,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E72" t="inlineStr"/>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -10382,6 +10589,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E73" t="inlineStr"/>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -10404,6 +10614,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E74" t="inlineStr"/>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -10418,7 +10631,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Plain crackers</t>
+          <t>Plain cracker</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -10426,6 +10639,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E75" t="inlineStr"/>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -10440,7 +10656,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Pretzels</t>
+          <t>Pretzel</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -10448,6 +10664,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E76" t="inlineStr"/>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -10462,7 +10681,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Original potato chips</t>
+          <t>Original potato chip</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -10470,6 +10689,7 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr">
         <is>
           <t>Y</t>
@@ -10502,6 +10722,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E78" t="inlineStr"/>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -10524,6 +10747,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E79" t="inlineStr"/>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -10538,7 +10764,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Cheese corn chips</t>
+          <t>Cheese corn chip</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -10546,6 +10772,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E80" t="inlineStr"/>
+      <c r="F80" t="inlineStr"/>
+      <c r="G80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -10560,7 +10789,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Choclate chip cookies</t>
+          <t>Choclate chip cookie</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -10568,6 +10797,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E81" t="inlineStr"/>
+      <c r="F81" t="inlineStr"/>
+      <c r="G81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -10590,6 +10822,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E82" t="inlineStr"/>
+      <c r="F82" t="inlineStr"/>
+      <c r="G82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -10604,7 +10839,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Chocolate coated biscuits</t>
+          <t>Chocolate coated biscuit</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -10612,6 +10847,7 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
         <is>
           <t>Y</t>
@@ -10636,7 +10872,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Chocolate cream wafers</t>
+          <t>Chocolate cream wafer</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -10644,11 +10880,9 @@
           <t>unhealthy</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -10671,11 +10905,13 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
+      <c r="G85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -10690,7 +10926,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Rice bubbles snack bars</t>
+          <t>Rice bubbles snack bar</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -10698,6 +10934,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -10712,7 +10951,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Flavoured rainbow Sticks</t>
+          <t>Flavoured rainbow stick</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -10720,6 +10959,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -10742,6 +10984,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -10769,6 +11014,7 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="F89" t="inlineStr"/>
       <c r="G89" t="inlineStr">
         <is>
           <t>Y</t>
@@ -10796,6 +11042,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -10810,7 +11059,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Grapes</t>
+          <t>Grape</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -10818,6 +11067,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -10840,6 +11092,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -10862,6 +11117,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -10884,6 +11142,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -10898,7 +11159,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>pears</t>
+          <t>Pear</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -10906,6 +11167,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -10920,7 +11184,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>pineapple</t>
+          <t>Pineapple</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -10928,6 +11192,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -10955,6 +11222,8 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -10969,7 +11238,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Bannanas</t>
+          <t>Banana</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -11006,7 +11275,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Oranges</t>
+          <t>Orange</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -11014,6 +11283,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -11036,6 +11308,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -11050,7 +11325,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Canned peaches</t>
+          <t>Canned peache</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -11058,6 +11333,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr"/>
+      <c r="G101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -11080,6 +11358,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr"/>
+      <c r="G102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -11102,6 +11383,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr"/>
+      <c r="G103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -11124,6 +11408,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr"/>
+      <c r="G104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -11138,7 +11425,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Banana Chips</t>
+          <t>Banana Chip</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -11146,6 +11433,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr"/>
+      <c r="G105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -11168,6 +11458,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -11190,6 +11483,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -11212,6 +11508,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr"/>
+      <c r="G108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -11234,6 +11533,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr"/>
+      <c r="G109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -11256,6 +11558,13 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -11278,6 +11587,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -11300,6 +11612,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr"/>
+      <c r="G112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -11314,7 +11629,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Pork sizzle steaks</t>
+          <t>Pork sizzle steak</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -11322,6 +11637,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr"/>
+      <c r="G113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -11344,6 +11662,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr"/>
+      <c r="G114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -11366,6 +11687,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -11380,7 +11704,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Chicken breast fillets</t>
+          <t>Chicken breast fillet</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -11425,6 +11749,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr"/>
+      <c r="G117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -11447,6 +11774,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -11469,6 +11799,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -11491,6 +11824,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -11505,7 +11841,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Tuna steaks</t>
+          <t>Tuna steak</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -11513,6 +11849,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -11527,7 +11866,7 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Thin Bbq sausages</t>
+          <t>Thin Bbq sausage</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -11535,6 +11874,8 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr"/>
       <c r="G122" t="inlineStr">
         <is>
           <t>Y</t>
@@ -11554,7 +11895,7 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Beef sausages</t>
+          <t>Beef sausage</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -11562,6 +11903,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -11576,7 +11920,7 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Beef burgers patties</t>
+          <t>Beef burgers pattie</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -11584,6 +11928,8 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr"/>
       <c r="G124" t="inlineStr">
         <is>
           <t>Y</t>
@@ -11603,7 +11949,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Lamb burgers</t>
+          <t>Lamb burger</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -11611,6 +11957,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr"/>
+      <c r="G125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -11625,7 +11974,7 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Beef Bbq burgers</t>
+          <t>Beef Bbq burger</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -11633,6 +11982,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E126" t="inlineStr"/>
+      <c r="F126" t="inlineStr"/>
+      <c r="G126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -11647,7 +11999,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Kransky bites</t>
+          <t>Kransky bite</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -11655,6 +12007,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -11677,6 +12032,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E128" t="inlineStr"/>
+      <c r="F128" t="inlineStr"/>
+      <c r="G128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -11699,6 +12057,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr"/>
+      <c r="G129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -11721,6 +12082,8 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E130" t="inlineStr"/>
+      <c r="F130" t="inlineStr"/>
       <c r="G130" t="inlineStr">
         <is>
           <t>Y</t>
@@ -11748,6 +12111,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E131" t="inlineStr"/>
+      <c r="F131" t="inlineStr"/>
+      <c r="G131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -11770,11 +12136,7 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E132" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="E132" t="inlineStr"/>
       <c r="F132" t="inlineStr">
         <is>
           <t>Y</t>
@@ -11807,6 +12169,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E133" t="inlineStr"/>
+      <c r="F133" t="inlineStr"/>
+      <c r="G133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -11829,6 +12194,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E134" t="inlineStr"/>
+      <c r="F134" t="inlineStr"/>
+      <c r="G134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -11843,7 +12211,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Frozen Broccoli</t>
+          <t>Frozen broccoli</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -11856,6 +12224,8 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="F135" t="inlineStr"/>
+      <c r="G135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -11870,7 +12240,7 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Frozen Vegetable Mix</t>
+          <t>Frozen vegetable mix</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -11878,6 +12248,13 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr"/>
+      <c r="G136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -11892,7 +12269,7 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Frozen Cauliflower</t>
+          <t>Frozen cauliflower</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -11900,6 +12277,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E137" t="inlineStr"/>
+      <c r="F137" t="inlineStr"/>
+      <c r="G137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -11922,6 +12302,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E138" t="inlineStr"/>
+      <c r="F138" t="inlineStr"/>
+      <c r="G138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -11936,7 +12319,7 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Frozen Beans</t>
+          <t>Frozen beans</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -11944,6 +12327,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E139" t="inlineStr"/>
+      <c r="F139" t="inlineStr"/>
+      <c r="G139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -11958,7 +12344,7 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>Chinese Stir Fry Mix Veg</t>
+          <t>Chinese stir fry mix veg</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -11966,6 +12352,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E140" t="inlineStr"/>
+      <c r="F140" t="inlineStr"/>
+      <c r="G140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -11980,7 +12369,7 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Frozen Carrots</t>
+          <t>Frozen carrots</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
@@ -11988,6 +12377,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E141" t="inlineStr"/>
+      <c r="F141" t="inlineStr"/>
+      <c r="G141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -12002,7 +12394,7 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Flavoured Iceblocks</t>
+          <t>Flavoured iceblocks</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
@@ -12010,11 +12402,13 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E142" t="inlineStr"/>
       <c r="F142" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
+      <c r="G142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -12037,6 +12431,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E143" t="inlineStr"/>
+      <c r="F143" t="inlineStr"/>
+      <c r="G143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -12059,11 +12456,13 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E144" t="inlineStr"/>
       <c r="F144" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
+      <c r="G144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -12086,6 +12485,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E145" t="inlineStr"/>
+      <c r="F145" t="inlineStr"/>
+      <c r="G145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -12108,6 +12510,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E146" t="inlineStr"/>
+      <c r="F146" t="inlineStr"/>
+      <c r="G146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -12122,7 +12527,7 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Chocolate Bavarian</t>
+          <t>Chocolate bavarian</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
@@ -12130,6 +12535,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E147" t="inlineStr"/>
+      <c r="F147" t="inlineStr"/>
+      <c r="G147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -12152,6 +12560,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E148" t="inlineStr"/>
+      <c r="F148" t="inlineStr"/>
+      <c r="G148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -12174,6 +12585,17 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E149" t="inlineStr"/>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -12188,7 +12610,7 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Meatlovers Pizza</t>
+          <t>Meatlovers pizza</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
@@ -12196,6 +12618,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E150" t="inlineStr"/>
+      <c r="F150" t="inlineStr"/>
+      <c r="G150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -12218,6 +12643,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E151" t="inlineStr"/>
+      <c r="F151" t="inlineStr"/>
+      <c r="G151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -12240,6 +12668,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E152" t="inlineStr"/>
+      <c r="F152" t="inlineStr"/>
+      <c r="G152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -12262,6 +12693,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E153" t="inlineStr"/>
+      <c r="F153" t="inlineStr"/>
+      <c r="G153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -12276,7 +12710,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Cheese &amp; Bacon Pizza</t>
+          <t>Cheese &amp; bacon pizza</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
@@ -12284,6 +12718,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E154" t="inlineStr"/>
+      <c r="F154" t="inlineStr"/>
+      <c r="G154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -12298,7 +12735,7 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Hawaiin Pizza</t>
+          <t>Hawaiin pizza</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
@@ -12335,7 +12772,7 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Puff Pastry Sheets</t>
+          <t>Puff pastry sheet</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
@@ -12343,6 +12780,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E156" t="inlineStr"/>
+      <c r="F156" t="inlineStr"/>
+      <c r="G156" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -12365,6 +12805,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E157" t="inlineStr"/>
+      <c r="F157" t="inlineStr"/>
+      <c r="G157" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -12379,7 +12822,7 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Beef Curry Puff</t>
+          <t>Beef curry puff</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
@@ -12387,6 +12830,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E158" t="inlineStr"/>
+      <c r="F158" t="inlineStr"/>
+      <c r="G158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -12401,7 +12847,7 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Quiche Cheese &amp; Bacon</t>
+          <t>Quiche cheese &amp; bacon</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
@@ -12409,6 +12855,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E159" t="inlineStr"/>
+      <c r="F159" t="inlineStr"/>
+      <c r="G159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -12423,7 +12872,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Dim Sim</t>
+          <t>Dim sim</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
@@ -12431,6 +12880,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E160" t="inlineStr"/>
+      <c r="F160" t="inlineStr"/>
+      <c r="G160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -12458,6 +12910,8 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="F161" t="inlineStr"/>
+      <c r="G161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -12480,6 +12934,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E162" t="inlineStr"/>
+      <c r="F162" t="inlineStr"/>
+      <c r="G162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -12502,6 +12959,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E163" t="inlineStr"/>
+      <c r="F163" t="inlineStr"/>
+      <c r="G163" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -12524,6 +12984,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E164" t="inlineStr"/>
+      <c r="F164" t="inlineStr"/>
+      <c r="G164" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -12546,6 +13009,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E165" t="inlineStr"/>
+      <c r="F165" t="inlineStr"/>
+      <c r="G165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -12560,7 +13026,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Tortillas</t>
+          <t>Tortilla</t>
         </is>
       </c>
       <c r="D166" t="inlineStr">
@@ -12568,6 +13034,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E166" t="inlineStr"/>
+      <c r="F166" t="inlineStr"/>
+      <c r="G166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -12590,6 +13059,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E167" t="inlineStr"/>
+      <c r="F167" t="inlineStr"/>
+      <c r="G167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -12612,6 +13084,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E168" t="inlineStr"/>
+      <c r="F168" t="inlineStr"/>
+      <c r="G168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -12639,6 +13114,8 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="F169" t="inlineStr"/>
+      <c r="G169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -12661,6 +13138,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E170" t="inlineStr"/>
+      <c r="F170" t="inlineStr"/>
+      <c r="G170" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -12675,7 +13155,7 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Glass noodles</t>
+          <t>Glass noodle</t>
         </is>
       </c>
       <c r="D171" t="inlineStr">
@@ -12683,6 +13163,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E171" t="inlineStr"/>
+      <c r="F171" t="inlineStr"/>
+      <c r="G171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -12705,6 +13188,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E172" t="inlineStr"/>
+      <c r="F172" t="inlineStr"/>
+      <c r="G172" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -12727,6 +13213,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E173" t="inlineStr"/>
+      <c r="F173" t="inlineStr"/>
+      <c r="G173" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -12749,6 +13238,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E174" t="inlineStr"/>
+      <c r="F174" t="inlineStr"/>
+      <c r="G174" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -12763,7 +13255,7 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Chick peas</t>
+          <t>Chickpeas</t>
         </is>
       </c>
       <c r="D175" t="inlineStr">
@@ -12771,6 +13263,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E175" t="inlineStr"/>
+      <c r="F175" t="inlineStr"/>
+      <c r="G175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -12793,6 +13288,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E176" t="inlineStr"/>
+      <c r="F176" t="inlineStr"/>
+      <c r="G176" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -12815,6 +13313,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E177" t="inlineStr"/>
+      <c r="F177" t="inlineStr"/>
+      <c r="G177" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -12837,6 +13338,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E178" t="inlineStr"/>
+      <c r="F178" t="inlineStr"/>
+      <c r="G178" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -12859,6 +13363,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E179" t="inlineStr"/>
+      <c r="F179" t="inlineStr"/>
+      <c r="G179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -12881,6 +13388,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E180" t="inlineStr"/>
+      <c r="F180" t="inlineStr"/>
+      <c r="G180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -12903,16 +13413,9 @@
           <t>healthy</t>
         </is>
       </c>
-      <c r="E181" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="F181" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="E181" t="inlineStr"/>
+      <c r="F181" t="inlineStr"/>
+      <c r="G181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -12935,6 +13438,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E182" t="inlineStr"/>
+      <c r="F182" t="inlineStr"/>
+      <c r="G182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -12949,7 +13455,7 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Unsalted mixed nuts</t>
+          <t>Unsalted mixed nut</t>
         </is>
       </c>
       <c r="D183" t="inlineStr">
@@ -12957,6 +13463,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E183" t="inlineStr"/>
+      <c r="F183" t="inlineStr"/>
+      <c r="G183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -12971,7 +13480,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Unsalted cashews</t>
+          <t>Unsalted cashew</t>
         </is>
       </c>
       <c r="D184" t="inlineStr">
@@ -12979,6 +13488,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E184" t="inlineStr"/>
+      <c r="F184" t="inlineStr"/>
+      <c r="G184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -13006,6 +13518,8 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="F185" t="inlineStr"/>
+      <c r="G185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -13028,6 +13542,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E186" t="inlineStr"/>
+      <c r="F186" t="inlineStr"/>
+      <c r="G186" t="inlineStr"/>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -13050,6 +13567,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E187" t="inlineStr"/>
+      <c r="F187" t="inlineStr"/>
+      <c r="G187" t="inlineStr"/>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -13072,6 +13592,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E188" t="inlineStr"/>
+      <c r="F188" t="inlineStr"/>
+      <c r="G188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -13086,7 +13609,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Pumpkin seeds</t>
+          <t>Pumpkin seed</t>
         </is>
       </c>
       <c r="D189" t="inlineStr">
@@ -13094,6 +13617,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E189" t="inlineStr"/>
+      <c r="F189" t="inlineStr"/>
+      <c r="G189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -13108,7 +13634,7 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Black chia seeds</t>
+          <t>Black chia seed</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
@@ -13116,6 +13642,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E190" t="inlineStr"/>
+      <c r="F190" t="inlineStr"/>
+      <c r="G190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -13130,7 +13659,7 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Sunflower seeds</t>
+          <t>Sunflower seed</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
@@ -13138,6 +13667,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E191" t="inlineStr"/>
+      <c r="F191" t="inlineStr"/>
+      <c r="G191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -13152,7 +13684,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Walnuts</t>
+          <t>Walnut</t>
         </is>
       </c>
       <c r="D192" t="inlineStr">
@@ -13160,6 +13692,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E192" t="inlineStr"/>
+      <c r="F192" t="inlineStr"/>
+      <c r="G192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -13174,7 +13709,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Almonds</t>
+          <t>Almond</t>
         </is>
       </c>
       <c r="D193" t="inlineStr">
@@ -13182,6 +13717,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E193" t="inlineStr"/>
+      <c r="F193" t="inlineStr"/>
+      <c r="G193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -13204,6 +13742,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E194" t="inlineStr"/>
+      <c r="F194" t="inlineStr"/>
+      <c r="G194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -13226,6 +13767,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E195" t="inlineStr"/>
+      <c r="F195" t="inlineStr"/>
+      <c r="G195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -13248,6 +13792,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E196" t="inlineStr"/>
+      <c r="F196" t="inlineStr"/>
+      <c r="G196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -13270,6 +13817,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E197" t="inlineStr"/>
+      <c r="F197" t="inlineStr"/>
+      <c r="G197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -13297,16 +13847,8 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="F198" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="G198" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="F198" t="inlineStr"/>
+      <c r="G198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -13329,6 +13871,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E199" t="inlineStr"/>
+      <c r="F199" t="inlineStr"/>
+      <c r="G199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -13351,6 +13896,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E200" t="inlineStr"/>
+      <c r="F200" t="inlineStr"/>
+      <c r="G200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -13373,6 +13921,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E201" t="inlineStr"/>
+      <c r="F201" t="inlineStr"/>
+      <c r="G201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -13395,6 +13946,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E202" t="inlineStr"/>
+      <c r="F202" t="inlineStr"/>
+      <c r="G202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -13417,6 +13971,8 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E203" t="inlineStr"/>
+      <c r="F203" t="inlineStr"/>
       <c r="G203" t="inlineStr">
         <is>
           <t>Y</t>
@@ -13444,6 +14000,8 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E204" t="inlineStr"/>
+      <c r="F204" t="inlineStr"/>
       <c r="G204" t="inlineStr">
         <is>
           <t>Y</t>
@@ -13471,6 +14029,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E205" t="inlineStr"/>
+      <c r="F205" t="inlineStr"/>
+      <c r="G205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -13493,6 +14054,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E206" t="inlineStr"/>
+      <c r="F206" t="inlineStr"/>
+      <c r="G206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -13515,6 +14079,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E207" t="inlineStr"/>
+      <c r="F207" t="inlineStr"/>
+      <c r="G207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -13537,6 +14104,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E208" t="inlineStr"/>
+      <c r="F208" t="inlineStr"/>
+      <c r="G208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -13559,6 +14129,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E209" t="inlineStr"/>
+      <c r="F209" t="inlineStr"/>
+      <c r="G209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -13581,6 +14154,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E210" t="inlineStr"/>
+      <c r="F210" t="inlineStr"/>
+      <c r="G210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -13603,6 +14179,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E211" t="inlineStr"/>
+      <c r="F211" t="inlineStr"/>
+      <c r="G211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -13625,6 +14204,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E212" t="inlineStr"/>
+      <c r="F212" t="inlineStr"/>
+      <c r="G212" t="inlineStr"/>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -13647,6 +14229,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E213" t="inlineStr"/>
+      <c r="F213" t="inlineStr"/>
+      <c r="G213" t="inlineStr"/>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -13679,6 +14264,7 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="G214" t="inlineStr"/>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -13701,6 +14287,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E215" t="inlineStr"/>
+      <c r="F215" t="inlineStr"/>
+      <c r="G215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -13723,6 +14312,7 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E216" t="inlineStr"/>
       <c r="F216" t="inlineStr">
         <is>
           <t>Y</t>
@@ -13755,6 +14345,8 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E217" t="inlineStr"/>
+      <c r="F217" t="inlineStr"/>
       <c r="G217" t="inlineStr">
         <is>
           <t>Y</t>
@@ -13782,6 +14374,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E218" t="inlineStr"/>
+      <c r="F218" t="inlineStr"/>
+      <c r="G218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -13804,6 +14399,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E219" t="inlineStr"/>
+      <c r="F219" t="inlineStr"/>
+      <c r="G219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -13826,6 +14424,8 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E220" t="inlineStr"/>
+      <c r="F220" t="inlineStr"/>
       <c r="G220" t="inlineStr">
         <is>
           <t>Y</t>
@@ -13853,6 +14453,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E221" t="inlineStr"/>
+      <c r="F221" t="inlineStr"/>
+      <c r="G221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -13875,6 +14478,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E222" t="inlineStr"/>
+      <c r="F222" t="inlineStr"/>
+      <c r="G222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -13897,6 +14503,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E223" t="inlineStr"/>
+      <c r="F223" t="inlineStr"/>
+      <c r="G223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -13919,6 +14528,9 @@
           <t>unhealthy</t>
         </is>
       </c>
+      <c r="E224" t="inlineStr"/>
+      <c r="F224" t="inlineStr"/>
+      <c r="G224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -13941,6 +14553,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E225" t="inlineStr"/>
+      <c r="F225" t="inlineStr"/>
+      <c r="G225" t="inlineStr"/>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -13973,6 +14588,7 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="G226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -13995,6 +14611,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E227" t="inlineStr"/>
+      <c r="F227" t="inlineStr"/>
+      <c r="G227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -14009,7 +14628,7 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>tomatoes</t>
+          <t>Tomato</t>
         </is>
       </c>
       <c r="D228" t="inlineStr">
@@ -14027,6 +14646,7 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="G228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -14049,6 +14669,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E229" t="inlineStr"/>
+      <c r="F229" t="inlineStr"/>
+      <c r="G229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -14081,6 +14704,7 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="G230" t="inlineStr"/>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -14113,6 +14737,7 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="G231" t="inlineStr"/>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -14135,6 +14760,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E232" t="inlineStr"/>
+      <c r="F232" t="inlineStr"/>
+      <c r="G232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -14157,6 +14785,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E233" t="inlineStr"/>
+      <c r="F233" t="inlineStr"/>
+      <c r="G233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -14184,6 +14815,8 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="F234" t="inlineStr"/>
+      <c r="G234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -14206,6 +14839,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E235" t="inlineStr"/>
+      <c r="F235" t="inlineStr"/>
+      <c r="G235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -14228,6 +14864,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E236" t="inlineStr"/>
+      <c r="F236" t="inlineStr"/>
+      <c r="G236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -14250,6 +14889,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E237" t="inlineStr"/>
+      <c r="F237" t="inlineStr"/>
+      <c r="G237" t="inlineStr"/>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
@@ -14277,6 +14919,8 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="F238" t="inlineStr"/>
+      <c r="G238" t="inlineStr"/>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
@@ -14299,6 +14943,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E239" t="inlineStr"/>
+      <c r="F239" t="inlineStr"/>
+      <c r="G239" t="inlineStr"/>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
@@ -14321,6 +14968,9 @@
           <t>healthy</t>
         </is>
       </c>
+      <c r="E240" t="inlineStr"/>
+      <c r="F240" t="inlineStr"/>
+      <c r="G240" t="inlineStr"/>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
@@ -14353,6 +15003,7 @@
           <t>Y</t>
         </is>
       </c>
+      <c r="G241" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -16021,7 +16672,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B259"/>
+  <dimension ref="B1:B259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="56.28515625" bestFit="1" customWidth="1" min="2" max="2"/>
@@ -16167,7 +16818,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="B22" t="inlineStr">
         <is>
@@ -16371,7 +17021,6 @@
         </is>
       </c>
     </row>
-    <row r="51"/>
     <row r="52">
       <c r="B52" t="inlineStr">
         <is>
@@ -16470,7 +17119,6 @@
         </is>
       </c>
     </row>
-    <row r="66"/>
     <row r="67">
       <c r="B67" t="inlineStr">
         <is>
@@ -16681,7 +17329,6 @@
         </is>
       </c>
     </row>
-    <row r="97"/>
     <row r="98">
       <c r="B98" t="inlineStr">
         <is>
@@ -16829,7 +17476,6 @@
         </is>
       </c>
     </row>
-    <row r="119"/>
     <row r="120">
       <c r="B120" t="inlineStr">
         <is>
@@ -16991,7 +17637,6 @@
         </is>
       </c>
     </row>
-    <row r="143"/>
     <row r="144">
       <c r="B144" t="inlineStr">
         <is>
@@ -17307,7 +17952,6 @@
         </is>
       </c>
     </row>
-    <row r="189"/>
     <row r="190">
       <c r="B190" t="inlineStr">
         <is>
@@ -17455,7 +18099,6 @@
         </is>
       </c>
     </row>
-    <row r="211"/>
     <row r="212">
       <c r="B212" t="inlineStr">
         <is>
@@ -17659,7 +18302,6 @@
         </is>
       </c>
     </row>
-    <row r="241"/>
     <row r="242">
       <c r="B242" t="inlineStr">
         <is>

</xml_diff>